<commit_message>
Island accruals mappings and files changed
</commit_message>
<xml_diff>
--- a/data/isx_xlsx/HEIMAR.IC.xlsx
+++ b/data/isx_xlsx/HEIMAR.IC.xlsx
@@ -7032,7 +7032,10 @@
       <c r="P30" s="17">
         <v>1.11</v>
       </c>
-      <c r="Q30" s="16"/>
+      <c r="Q30" s="16">
+        <f>SUM(Q31,Q36)</f>
+        <v>3.08</v>
+      </c>
       <c r="R30" s="17">
         <v>5.63</v>
       </c>
@@ -7547,9 +7550,15 @@
       <c r="A46" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="16"/>
+      <c r="B46" s="15">
+        <v>367.83</v>
+      </c>
+      <c r="C46" s="15">
+        <v>436.32</v>
+      </c>
+      <c r="D46" s="15">
+        <v>281.34</v>
+      </c>
       <c r="E46" s="15">
         <v>542.32</v>
       </c>

</xml_diff>